<commit_message>
Auto-synced valid live SharePoint Excel binary
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,7 +1,3 @@
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">

</xml_diff>